<commit_message>
removed group policy to avoid antivisrus error
</commit_message>
<xml_diff>
--- a/Scripts/Config.xlsx
+++ b/Scripts/Config.xlsx
@@ -9,14 +9,15 @@
     <sheet name="Download" sheetId="2" r:id="rId3"/>
     <sheet name="PWAttributesList" sheetId="3" r:id="rId4"/>
     <sheet name="Federation" sheetId="4" r:id="rId5"/>
-    <sheet name="Lookups" sheetId="5" r:id="rId6"/>
+    <sheet name="WildcardSelection" sheetId="5" r:id="rId6"/>
+    <sheet name="Lookups" sheetId="6" r:id="rId7"/>
   </sheets>
   <calcPr fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="152">
   <si>
     <t>Parameter</t>
   </si>
@@ -66,7 +67,7 @@
     <t>SourceAcquisitionMode</t>
   </si>
   <si>
-    <t>Auto</t>
+    <t>Local</t>
   </si>
   <si>
     <t>Select Local, ProjectWise, or Auto. Auto supports a mixture of configured source rows.</t>
@@ -90,6 +91,9 @@
     <t>RunProcess</t>
   </si>
   <si>
+    <t>No</t>
+  </si>
+  <si>
     <t>Yes runs IFC processing when needed; No skips it; Force reprocesses all applicable IFC files.</t>
   </si>
   <si>
@@ -111,6 +115,15 @@
     <t>Yes uses change-based federation; No disables it; Force always rebuilds the federation.</t>
   </si>
   <si>
+    <t>FederationGroupingMethod</t>
+  </si>
+  <si>
+    <t>Wildcard Selection</t>
+  </si>
+  <si>
+    <t>Choose Naming Convention and Lookups or Wildcard Selection.</t>
+  </si>
+  <si>
     <t>IncludeUnmatchedFilesInFederatedModel</t>
   </si>
   <si>
@@ -165,9 +178,6 @@
     <t>NavisworksVisible</t>
   </si>
   <si>
-    <t>No</t>
-  </si>
-  <si>
     <t>Yes shows Navisworks while federation runs; No runs it in the background.</t>
   </si>
   <si>
@@ -219,7 +229,7 @@
     <t>MinState</t>
   </si>
   <si>
-    <t>C:\Users\GoodyGudarzian\DC\ACCDocs\X(AUS Server)\Link\Project Files\01 WIP\1</t>
+    <t>C:\Users\GoodyGudarzian\DC\ACCDocs\AUS\ProjectName\Project Files\01 WIP\</t>
   </si>
   <si>
     <t>*.ifc</t>
@@ -228,9 +238,6 @@
     <t>delete,Delete,WITHDRAWN</t>
   </si>
   <si>
-    <t>C:\Users\GoodyGudarzian\DC\ACCDocs\X(AUS Server)\Link\Project Files\01 WIP\2</t>
-  </si>
-  <si>
     <t>AttributeName</t>
   </si>
   <si>
@@ -330,6 +337,66 @@
     <t>WorkflowState</t>
   </si>
   <si>
+    <t>CustomAttributes.INFO_DC_PROJECT_STAGE</t>
+  </si>
+  <si>
+    <t>PROJECT_STAGE</t>
+  </si>
+  <si>
+    <t>CustomAttributes.WRE_OPERATION</t>
+  </si>
+  <si>
+    <t>WRE_OPERATION</t>
+  </si>
+  <si>
+    <t>CustomAttributes.TB_LINE_DISCIPLINE</t>
+  </si>
+  <si>
+    <t>TB_LINE_DISCIPLINE</t>
+  </si>
+  <si>
+    <t>CustomAttributes.TB_DISCIPLIN</t>
+  </si>
+  <si>
+    <t>TB_DISCIPLIN</t>
+  </si>
+  <si>
+    <t>CustomAttributes.DC_SUB_DISCIPLINE</t>
+  </si>
+  <si>
+    <t>DC_SUB_DISCIPLINE</t>
+  </si>
+  <si>
+    <t>CustomAttributes.PW_PACKAGE_NO</t>
+  </si>
+  <si>
+    <t>PW_PACKAGE_NO</t>
+  </si>
+  <si>
+    <t>CustomAttributes.INFO_TB_SUITABILITY</t>
+  </si>
+  <si>
+    <t>INFO_TB_SUITABILITY</t>
+  </si>
+  <si>
+    <t>CustomAttributes.TB_SUITABILITY</t>
+  </si>
+  <si>
+    <t>TB_SUITABILITY</t>
+  </si>
+  <si>
+    <t>CustomAttributes.TB_STATUS</t>
+  </si>
+  <si>
+    <t>TB_STATUS</t>
+  </si>
+  <si>
+    <t>CustomAttributes.INFO_TB_STATUS</t>
+  </si>
+  <si>
+    <t>INFO_TB_STATUS</t>
+  </si>
+  <si>
     <t>FieldNames</t>
   </si>
   <si>
@@ -357,13 +424,52 @@
     <t>Discipline/Sub</t>
   </si>
   <si>
-    <t>Discipline-Sub</t>
-  </si>
-  <si>
     <t>SequenceNumber</t>
   </si>
   <si>
     <t>FileExtension</t>
+  </si>
+  <si>
+    <t>Inclusions</t>
+  </si>
+  <si>
+    <t>Exclusions</t>
+  </si>
+  <si>
+    <t>ExportFileName</t>
+  </si>
+  <si>
+    <t>ReadFromOutputFolder</t>
+  </si>
+  <si>
+    <t>*ARC*.ifc</t>
+  </si>
+  <si>
+    <t>SX-MOD-PDE-100000.nwd</t>
+  </si>
+  <si>
+    <t>*-C*.ifc</t>
+  </si>
+  <si>
+    <t>SX-MOD-PDE-100001.nwd</t>
+  </si>
+  <si>
+    <t>*MFP*.ifc</t>
+  </si>
+  <si>
+    <t>SX-MOD-PDE-100003.nwd</t>
+  </si>
+  <si>
+    <t>*MHV*.ifc</t>
+  </si>
+  <si>
+    <t>SX-MOD-PDE-100004.nwd</t>
+  </si>
+  <si>
+    <t>SX-MOD-PDE-10000?.NWD</t>
+  </si>
+  <si>
+    <t>SX-MOD-PDE-000002.nwd</t>
   </si>
   <si>
     <t>Code</t>
@@ -441,8 +547,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Settings" displayName="Settings" ref="A1:C23" headerRowCount="1">
-  <autoFilter ref="A1:C23"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Settings" displayName="Settings" ref="A1:C24" headerRowCount="1">
+  <autoFilter ref="A1:C24"/>
   <tableColumns count="3">
     <tableColumn id="1" name="Parameter"/>
     <tableColumn id="2" name="Value"/>
@@ -453,8 +559,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Download" displayName="Download" ref="A1:G11" headerRowCount="1">
-  <autoFilter ref="A1:G11"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Download" displayName="Download" ref="A1:G10" headerRowCount="1">
+  <autoFilter ref="A1:G10"/>
   <tableColumns count="7">
     <tableColumn id="1" name="Run"/>
     <tableColumn id="2" name="ReadFolder"/>
@@ -469,8 +575,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="PWAttributesList" displayName="PWAttributesList" ref="A1:D17" headerRowCount="1">
-  <autoFilter ref="A1:D17"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="PWAttributesList" displayName="PWAttributesList" ref="A1:D27" headerRowCount="1">
+  <autoFilter ref="A1:D27"/>
   <tableColumns count="4">
     <tableColumn id="1" name="AttributeName"/>
     <tableColumn id="2" name="OutputName"/>
@@ -496,7 +602,20 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Lookups" displayName="Lookups" ref="A1:C2" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="WildcardSelection" displayName="WildcardSelection" ref="A1:D6" headerRowCount="1">
+  <autoFilter ref="A1:D6"/>
+  <tableColumns count="4">
+    <tableColumn id="1" name="Inclusions"/>
+    <tableColumn id="2" name="Exclusions"/>
+    <tableColumn id="3" name="ExportFileName"/>
+    <tableColumn id="4" name="ReadFromOutputFolder"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium6" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Lookups" displayName="Lookups" ref="A1:C2" headerRowCount="1">
   <autoFilter ref="A1:C2"/>
   <tableColumns count="3">
     <tableColumn id="1" name="Filename-Part"/>
@@ -509,7 +628,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="38.3433036804199" customWidth="1"/>
@@ -610,164 +729,175 @@
         <v>23</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>13</v>
+        <v>33</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>36</v>
+        <v>7</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>19</v>
+        <v>43</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>44</v>
+        <v>19</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>19</v>
+        <v>48</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>49</v>
+        <v>19</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>52</v>
+        <v>24</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="s">
+      <c r="A21" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="B21" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="C21" s="5" t="s">
+      <c r="B21" s="4" t="s">
         <v>55</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="B23" s="5">
+        <v>59</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C23" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="C23" s="5" t="s">
-        <v>59</v>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="B24" s="5">
+        <v>60</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>62</v>
       </c>
     </row>
   </sheetData>
@@ -780,11 +910,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="9.140625" customWidth="1"/>
-    <col min="2" max="2" width="74.116828918457" customWidth="1"/>
+    <col min="2" max="2" width="72.4257049560547" customWidth="1"/>
     <col min="3" max="3" width="11.2497501373291" customWidth="1"/>
     <col min="4" max="4" width="25.7544898986816" customWidth="1"/>
     <col min="5" max="5" width="13.2887191772461" customWidth="1"/>
@@ -794,25 +924,25 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="E1" s="0" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="F1" s="0" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="G1" s="0" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2">
@@ -820,13 +950,13 @@
         <v>13</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E2" s="0" t="s">
         <v>13</v>
@@ -840,22 +970,22 @@
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>70</v>
+        <v>19</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>68</v>
+        <v>19</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>69</v>
+        <v>19</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="G3" s="0" t="s">
         <v>19</v>
@@ -863,7 +993,7 @@
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="B4" s="0" t="s">
         <v>19</v>
@@ -875,10 +1005,10 @@
         <v>19</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="G4" s="0" t="s">
         <v>19</v>
@@ -886,7 +1016,7 @@
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="B5" s="0" t="s">
         <v>19</v>
@@ -898,10 +1028,10 @@
         <v>19</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="G5" s="0" t="s">
         <v>19</v>
@@ -909,7 +1039,7 @@
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="B6" s="0" t="s">
         <v>19</v>
@@ -921,10 +1051,10 @@
         <v>19</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="G6" s="0" t="s">
         <v>19</v>
@@ -932,7 +1062,7 @@
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="B7" s="0" t="s">
         <v>19</v>
@@ -944,10 +1074,10 @@
         <v>19</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="G7" s="0" t="s">
         <v>19</v>
@@ -955,7 +1085,7 @@
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="B8" s="0" t="s">
         <v>19</v>
@@ -967,10 +1097,10 @@
         <v>19</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="F8" s="0" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="G8" s="0" t="s">
         <v>19</v>
@@ -978,7 +1108,7 @@
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="B9" s="0" t="s">
         <v>19</v>
@@ -990,10 +1120,10 @@
         <v>19</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="F9" s="0" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="G9" s="0" t="s">
         <v>19</v>
@@ -1001,7 +1131,7 @@
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="B10" s="0" t="s">
         <v>19</v>
@@ -1013,35 +1143,12 @@
         <v>19</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="F10" s="0" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="0" t="s">
-        <v>49</v>
-      </c>
-      <c r="B11" s="0" t="s">
-        <v>19</v>
-      </c>
-      <c r="C11" s="0" t="s">
-        <v>19</v>
-      </c>
-      <c r="D11" s="0" t="s">
-        <v>19</v>
-      </c>
-      <c r="E11" s="0" t="s">
-        <v>49</v>
-      </c>
-      <c r="F11" s="0" t="s">
-        <v>49</v>
-      </c>
-      <c r="G11" s="0" t="s">
         <v>19</v>
       </c>
     </row>
@@ -1055,10 +1162,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="24.9493389129639" customWidth="1"/>
+    <col min="1" max="1" width="40.9531478881836" customWidth="1"/>
     <col min="2" max="2" width="26.5985202789307" customWidth="1"/>
     <col min="3" max="3" width="15.7266845703125" customWidth="1"/>
     <col min="4" max="4" width="13.4411563873291" customWidth="1"/>
@@ -1066,24 +1173,24 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C2" s="0" t="s">
         <v>13</v>
@@ -1094,24 +1201,24 @@
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C3" s="0" t="s">
         <v>13</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C4" s="0" t="s">
         <v>13</v>
@@ -1122,13 +1229,13 @@
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="D5" s="0" t="s">
         <v>13</v>
@@ -1136,10 +1243,10 @@
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C6" s="0" t="s">
         <v>13</v>
@@ -1150,52 +1257,52 @@
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C7" s="0" t="s">
         <v>13</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C8" s="0" t="s">
         <v>13</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C9" s="0" t="s">
         <v>13</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C10" s="0" t="s">
         <v>13</v>
@@ -1206,24 +1313,24 @@
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C11" s="0" t="s">
         <v>13</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C12" s="0" t="s">
         <v>13</v>
@@ -1234,10 +1341,10 @@
     </row>
     <row r="13">
       <c r="A13" s="0" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C13" s="0" t="s">
         <v>13</v>
@@ -1248,10 +1355,10 @@
     </row>
     <row r="14">
       <c r="A14" s="0" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C14" s="0" t="s">
         <v>13</v>
@@ -1262,10 +1369,10 @@
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C15" s="0" t="s">
         <v>13</v>
@@ -1276,10 +1383,10 @@
     </row>
     <row r="16">
       <c r="A16" s="0" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B16" s="0" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C16" s="0" t="s">
         <v>13</v>
@@ -1290,16 +1397,156 @@
     </row>
     <row r="17">
       <c r="A17" s="0" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B17" s="0" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C17" s="0" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="D17" s="0" t="s">
-        <v>49</v>
+        <v>24</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="s">
+        <v>106</v>
+      </c>
+      <c r="B18" s="0" t="s">
+        <v>107</v>
+      </c>
+      <c r="C18" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="D18" s="0" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="s">
+        <v>108</v>
+      </c>
+      <c r="B19" s="0" t="s">
+        <v>109</v>
+      </c>
+      <c r="C19" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="D19" s="0" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="B20" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="C20" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="D20" s="0" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="s">
+        <v>112</v>
+      </c>
+      <c r="B21" s="0" t="s">
+        <v>113</v>
+      </c>
+      <c r="C21" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="D21" s="0" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="s">
+        <v>114</v>
+      </c>
+      <c r="B22" s="0" t="s">
+        <v>115</v>
+      </c>
+      <c r="C22" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="D22" s="0" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="s">
+        <v>116</v>
+      </c>
+      <c r="B23" s="0" t="s">
+        <v>117</v>
+      </c>
+      <c r="C23" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="D23" s="0" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="s">
+        <v>118</v>
+      </c>
+      <c r="B24" s="0" t="s">
+        <v>119</v>
+      </c>
+      <c r="C24" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24" s="0" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="s">
+        <v>120</v>
+      </c>
+      <c r="B25" s="0" t="s">
+        <v>121</v>
+      </c>
+      <c r="C25" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="D25" s="0" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="B26" s="0" t="s">
+        <v>123</v>
+      </c>
+      <c r="C26" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="D26" s="0" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="s">
+        <v>124</v>
+      </c>
+      <c r="B27" s="0" t="s">
+        <v>125</v>
+      </c>
+      <c r="C27" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="D27" s="0" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -1324,24 +1571,24 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>104</v>
+        <v>126</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>105</v>
+        <v>127</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>106</v>
+        <v>128</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E1" s="0" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>107</v>
+        <v>129</v>
       </c>
       <c r="B2" s="0">
         <v>1</v>
@@ -1350,15 +1597,15 @@
         <v>0</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>107</v>
+        <v>129</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>108</v>
+        <v>130</v>
       </c>
       <c r="B3" s="0">
         <v>2</v>
@@ -1367,15 +1614,15 @@
         <v>1</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>108</v>
+        <v>130</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>109</v>
+        <v>131</v>
       </c>
       <c r="B4" s="0">
         <v>3</v>
@@ -1384,15 +1631,15 @@
         <v>0</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>109</v>
+        <v>131</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>110</v>
+        <v>132</v>
       </c>
       <c r="B5" s="0">
         <v>4</v>
@@ -1401,15 +1648,15 @@
         <v>0</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>110</v>
+        <v>132</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>111</v>
+        <v>133</v>
       </c>
       <c r="B6" s="0">
         <v>5</v>
@@ -1418,32 +1665,32 @@
         <v>0</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>111</v>
+        <v>133</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>112</v>
+        <v>134</v>
       </c>
       <c r="B7" s="0">
         <v>6</v>
       </c>
       <c r="C7" s="0">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>113</v>
+        <v>134</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>114</v>
+        <v>135</v>
       </c>
       <c r="B8" s="0">
         <v>7</v>
@@ -1452,27 +1699,27 @@
         <v>0</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>114</v>
+        <v>135</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>115</v>
+        <v>136</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>115</v>
+        <v>136</v>
       </c>
       <c r="C9" s="0">
         <v>0</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>115</v>
+        <v>136</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -1484,6 +1731,109 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="25.2613735198975" customWidth="1"/>
+    <col min="2" max="2" width="12.6472568511963" customWidth="1"/>
+    <col min="3" max="3" width="24.5237426757813" customWidth="1"/>
+    <col min="4" max="4" width="24.5403919219971" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="0" t="s">
+        <v>137</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>138</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>139</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="s">
+        <v>141</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>142</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="s">
+        <v>143</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>144</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="s">
+        <v>145</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>146</v>
+      </c>
+      <c r="D4" s="0" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="s">
+        <v>147</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" s="0" t="s">
+        <v>148</v>
+      </c>
+      <c r="D5" s="0" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="s">
+        <v>149</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="0" t="s">
+        <v>150</v>
+      </c>
+      <c r="D6" s="0" t="s">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <headerFooter/>
+  <tableParts>
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1495,13 +1845,13 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>105</v>
+        <v>127</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>116</v>
+        <v>151</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2">

</xml_diff>